<commit_message>
chore: update Instagram report 2026-09-18 06:27
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/2026-09-18.xlsx
+++ b/instagram-daily-checker/reports/2026-09-18.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-18 05:53:48</t>
+          <t>取得日時：2026-09-18 06:27:17</t>
         </is>
       </c>
     </row>
@@ -1509,19 +1509,19 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>93</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">

</xml_diff>